<commit_message>
new recipe option added
</commit_message>
<xml_diff>
--- a/ERP_Estimate.xlsx
+++ b/ERP_Estimate.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,20 +46,36 @@
       <sz val="12"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="002F5597"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -73,12 +89,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF1DE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,23 +128,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00D3D3D3"/>
       </left>
       <right style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00D3D3D3"/>
       </right>
       <top style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00D3D3D3"/>
       </top>
       <bottom style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00D3D3D3"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -119,17 +155,31 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -582,7 +632,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -612,7 +662,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -642,7 +692,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -672,7 +722,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.013</v>
+        <v>0.057</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -693,24 +743,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0504130432</t>
+          <t>0101011311</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>G.I. Stay Set HT (1830X20MM) WRKG LD-7900KG</t>
+          <t>M.S Angle 65X65X6mm</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1</v>
+        <v>0.022</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>795.83</v>
+        <v>108667.24</v>
       </c>
       <c r="G10" s="4">
         <f>ROUND(D10*F10, 2)</f>
@@ -723,16 +773,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0503050711</t>
+          <t>0103011511</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>G.I. Stay Wire 7/3.15MM (10 SWG)</t>
+          <t>M.S Flat 65X6 mm</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.006</v>
+        <v>0.053</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -740,7 +790,7 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>142310.93</v>
+        <v>117493.74</v>
       </c>
       <c r="G11" s="4">
         <f>ROUND(D11*F11, 2)</f>
@@ -753,16 +803,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0508040841</t>
+          <t>0508011141</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Porcelain Guy Insulator HT</t>
+          <t>11 KV Polymer Composite Pin Insulator 5KN 320MM CD</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -770,7 +820,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>52.24</v>
+        <v>243.79</v>
       </c>
       <c r="G12" s="4">
         <f>ROUND(D12*F12, 2)</f>
@@ -783,24 +833,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0101011311</t>
+          <t>0504130432</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M.S Angle 65X65X6mm</t>
+          <t>G.I. Stay Set HT (1830X20MM) WRKG LD-7900KG</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.022</v>
+        <v>9</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>SET</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>108667.24</v>
+        <v>795.83</v>
       </c>
       <c r="G13" s="4">
         <f>ROUND(D13*F13, 2)</f>
@@ -813,16 +863,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0103011511</t>
+          <t>0503050711</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>M.S Flat 65X6 mm</t>
+          <t>G.I. Stay Wire 7/3.15MM (10 SWG)</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.003</v>
+        <v>0.056</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -830,7 +880,7 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>117493.74</v>
+        <v>142310.93</v>
       </c>
       <c r="G14" s="4">
         <f>ROUND(D14*F14, 2)</f>
@@ -843,16 +893,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0508030541</t>
+          <t>0508040841</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 KV Polymer Composite Disc Insulator 45KN</t>
+          <t>Porcelain Guy Insulator HT</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -860,7 +910,7 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>183.15</v>
+        <v>52.24</v>
       </c>
       <c r="G15" s="4">
         <f>ROUND(D15*F15, 2)</f>
@@ -873,24 +923,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0504010132</t>
+          <t>0508030541</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Composite Hardware Fittings for ACSR Weasel/Rabbit (30/50SQMM)</t>
+          <t>11 KV Polymer Composite Disc Insulator 45KN</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3.09</v>
+        <v>12</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>327.83</v>
+        <v>183.15</v>
       </c>
       <c r="G16" s="4">
         <f>ROUND(D16*F16, 2)</f>
@@ -903,24 +953,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0503010711</t>
+          <t>0504010132</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>G.I. Wire 4 MM (8 SWG)</t>
+          <t>Composite Hardware Fittings for ACSR Weasel/Rabbit (30/50SQMM)</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.004</v>
+        <v>12.36</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>SET</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>137360.98</v>
+        <v>327.83</v>
       </c>
       <c r="G17" s="4">
         <f>ROUND(D17*F17, 2)</f>
@@ -933,24 +983,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0502010921</t>
+          <t>0102010611</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ACSR Conductor 50SQMM (Rabbit)</t>
+          <t>M.S Channel 75X40 mm</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.124</v>
+        <v>0.099</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KM</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>62290.12</v>
+        <v>110043.09</v>
       </c>
       <c r="G18" s="4">
         <f>ROUND(D18*F18, 2)</f>
@@ -958,96 +1008,209 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="A19" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0502010921</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Material Base Total</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+          <t>ACSR Conductor 50SQMM (Rabbit)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>62290.12</v>
+      </c>
       <c r="G19" s="4">
-        <f>ROUND(SUM(G6:G18), 2)</f>
+        <f>ROUND(D19*F19, 2)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="A20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0309010841</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Add: Escalation @ 5% for FY 26-27</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+          <t>Lightning Arrestor 12KV 5KA Porcelain Gapless Type 11KV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>524.23</v>
+      </c>
       <c r="G20" s="4">
-        <f>ROUND((G19)*0.05, 2)</f>
+        <f>ROUND(D20*F20, 2)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="A21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0304010532</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Add: Sundries @ 5%</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+          <t>T.P.G.O. Isolator 11KV 200 AMP</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>10384.98</v>
+      </c>
       <c r="G21" s="4">
-        <f>ROUND((G19+G20)*0.05, 2)</f>
+        <f>ROUND(D21*F21, 2)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL MATERIAL COST (A)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" s="5">
-        <f>ROUND(G19+G20+G21, 2)</f>
+      <c r="A22" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0912011441</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>G.I. Turn Buckle 18x5/8"</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>182.36</v>
+      </c>
+      <c r="G22" s="4">
+        <f>ROUND(D22*F22, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0501017821</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CABLE (PVC 1.1KV GRADE) 4CX25SQMM</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>229429.95</v>
+      </c>
+      <c r="G23" s="4">
+        <f>ROUND(D23*F23, 2)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>B. ERECTION / LABOR</t>
-        </is>
+      <c r="A24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0102010911</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>M.S Channel 100X50 mm</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>109813.95</v>
+      </c>
+      <c r="G24" s="4">
+        <f>ROUND(D24*F24, 2)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0503010711</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Erection of 9MTR PCC Pole (HT) Without Painted</t>
+          <t>G.I. Wire 4 MM (8 SWG)</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>1</v>
+        <v>0.012</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>2620</v>
+        <v>137360.98</v>
       </c>
       <c r="G25" s="4">
         <f>ROUND(D25*F25, 2)</f>
@@ -1055,233 +1218,128 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>2</v>
-      </c>
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Pole GIS Survey</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>31</v>
-      </c>
+          <t>Material Base Total</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" s="4">
-        <f>ROUND(D26*F26, 2)</f>
+        <f>ROUND(SUM(G6:G25), 2)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
-        <v>3</v>
-      </c>
+      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fixing of Caution Board</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n">
-        <v>24</v>
-      </c>
+          <t>Add: Escalation @ 5% for FY 24-25</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" s="4">
-        <f>ROUND(D27*F27, 2)</f>
+        <f>ROUND((G26)*0.05, 2)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>4</v>
-      </c>
+      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Earthing Complete</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n">
-        <v>313</v>
-      </c>
+          <t>Add: Escalation @ 5% for FY 25-26</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" s="4">
-        <f>ROUND(D28*F28, 2)</f>
+        <f>ROUND((G26+G27)*0.05, 2)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
-        <v>5</v>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>H.T. Stay Set Complete Labour</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>SET</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n">
-        <v>641</v>
-      </c>
+          <t>Add: Escalation @ 5% for FY 26-27</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" s="4">
-        <f>ROUND(D29*F29, 2)</f>
+        <f>ROUND((G26+G27+G28)*0.05, 2)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
-        <v>6</v>
-      </c>
+      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fabrication &amp; Fixing of CG Bracket Single Pole</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="n">
-        <v>237</v>
-      </c>
+          <t>Add: Sundries @ 5%</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" s="4">
-        <f>ROUND(D30*F30, 2)</f>
+        <f>ROUND((G26+G27+G28+G29)*0.05, 2)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>7</v>
-      </c>
+      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Fixing of 11KV Disc Insulator with Strain Hardware</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="G31" s="4">
-        <f>ROUND(D31*F31, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>8</v>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Fixing of Solid Tee-off Bracket on Double Pole</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>1483</v>
-      </c>
-      <c r="G32" s="4">
-        <f>ROUND(D32*F32, 2)</f>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL MATERIAL COST (A)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" s="5">
+        <f>ROUND(G26+G27+G28+G29+G30, 2)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
-        <v>9</v>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Fixing Cross Lacing Wire</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G33" s="4">
-        <f>ROUND(D33*F33, 2)</f>
-        <v/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>B. ERECTION / LABOR</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Stringing &amp; Sagging ACSR 50SQMM 3 Wire</t>
+          <t>Erection of 9MTR PCC Pole (HT) Without Painted</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.04</v>
+        <v>2</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KM</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>8289</v>
+        <v>2620</v>
       </c>
       <c r="G34" s="4">
         <f>ROUND(D34*F34, 2)</f>
@@ -1290,24 +1348,24 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Survey for H.T.O.H Line</t>
+          <t>Pole GIS Survey</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>KM</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>2761</v>
+        <v>31</v>
       </c>
       <c r="G35" s="4">
         <f>ROUND(D35*F35, 2)</f>
@@ -1315,105 +1373,469 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="n">
+        <v>3</v>
+      </c>
       <c r="B36" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL LABOR COST (B)</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" s="5">
-        <f>ROUND(SUM(G25:G35), 2)</f>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fixing of Caution Board</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G36" s="4">
+        <f>ROUND(D36*F36, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Earthing Complete</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>313</v>
+      </c>
+      <c r="G37" s="4">
+        <f>ROUND(D37*F37, 2)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>C. OVERHEADS &amp; TAXES</t>
-        </is>
+      <c r="A38" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fabrication &amp; Fixing of CG Bracket Single Pole</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>237</v>
+      </c>
+      <c r="G38" s="4">
+        <f>ROUND(D38*F38, 2)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
+      <c r="A39" t="n">
+        <v>6</v>
+      </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Supervision @ 10% on (A+B)</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
+          <t>Fixing of 11KV Pin Insulator</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>63</v>
+      </c>
       <c r="G39" s="4">
-        <f>ROUND((G22+G36)*0.1, 2)</f>
+        <f>ROUND(D39*F39, 2)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" t="n">
+        <v>7</v>
+      </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GST @ 18% on Labour only</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
+          <t>H.T. Stay Set Complete Labour</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>641</v>
+      </c>
       <c r="G40" s="4">
-        <f>ROUND(G36*0.18, 2)</f>
+        <f>ROUND(D40*F40, 2)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" t="n">
+        <v>8</v>
+      </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Sub-Total</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+          <t>Fixing of 11KV Disc Insulator with Strain Hardware</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>65</v>
+      </c>
       <c r="G41" s="4">
-        <f>ROUND(G22+G36+G39+G40, 2)</f>
+        <f>ROUND(D41*F41, 2)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
+      <c r="A42" t="n">
+        <v>9</v>
+      </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
+          <t>Erection of DP Structure 9MTR PCC Pole HT</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>9438</v>
+      </c>
+      <c r="G42" s="4">
+        <f>ROUND(D42*F42, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Erection of S/S DP Structure 9MTR PCC Pole Without Painted</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>13169</v>
+      </c>
+      <c r="G43" s="4">
+        <f>ROUND(D43*F43, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>11</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Fixing of 11KV Lightning Arrestor on Structure</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>339</v>
+      </c>
+      <c r="G44" s="4">
+        <f>ROUND(D44*F44, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>12</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Fixing of 11KV TPGO Isolator on S/Stn Structure</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>1193</v>
+      </c>
+      <c r="G45" s="4">
+        <f>ROUND(D45*F45, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>13</v>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Fixing of Neutral Earthing of DTR with G</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>3816</v>
+      </c>
+      <c r="G46" s="4">
+        <f>ROUND(D46*F46, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>14</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Fixing Cross Lacing Wire</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G47" s="4">
+        <f>ROUND(D47*F47, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>15</v>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Stringing &amp; Sagging ACSR 50SQMM 3 Wire</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>8289</v>
+      </c>
+      <c r="G48" s="4">
+        <f>ROUND(D48*F48, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>16</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Survey for H.T.O.H Line</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>2761</v>
+      </c>
+      <c r="G49" s="4">
+        <f>ROUND(D49*F49, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL LABOR COST (B)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" s="5">
+        <f>ROUND(SUM(G34:G49), 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>C. OVERHEADS &amp; TAXES</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Supervision @ 10% on (A+B)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" s="4">
+        <f>ROUND((G31+G50)*0.1, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GST @ 18% on Labour only</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" s="4">
+        <f>ROUND(G50*0.18, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sub-Total</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" s="4">
+        <f>ROUND(G31+G50+G53+G54, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
           <t>Add: Cess @ 1% on (Mat+Lab+Sup)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" s="4">
-        <f>ROUND((G22+G36+G39)*0.01, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" s="4">
+        <f>ROUND((G31+G50+G53)*0.01, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" s="7">
-        <f>ROUND(G41+G42, 2)</f>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" s="7">
+        <f>ROUND(G55+G56, 2)</f>
         <v/>
       </c>
     </row>
@@ -1433,373 +1855,586 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
           <t>IRON CALCULATION BREAKUP</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Steel quantities from rule-engine + 3% wastage &amp; sag</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>M.S. Angle (65X65X6mm)</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
+          <t>DTR Substation Iron (1 nos on canvas)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Lgth(m)</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Total(m)</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Wt(kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Length (m)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Total (m)</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Wt (kg)</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>Cradle Guard (CG) Bracket on Pole</t>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>M.S Channel 75X40 mm</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11">
+        <f>2.375</f>
+        <v/>
+      </c>
+      <c r="E4" s="11">
+        <f>C4*D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="G4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="11" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>22.04</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Add: Wastage + Sag @ 3%</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
-      <c r="E5" s="11" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Total (incl. 3% wastage &amp; sag)</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="13" t="n">
-        <v>3.914</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>22.7</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>M.S. Flat (65X6mm)</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>M.S Channel 100X50 mm</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="13">
+        <f>2.5</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="G5" s="14" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Channel subtotal</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="16">
+        <f>SUM(E4:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>SUM(F4:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="15" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>M.S Angle 65X65X6mm (Structure Support)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="11">
+        <f>1.75</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="G7" s="12" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>M.S Angle 65X65X6mm (Transformer Base Bracing)</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="13">
+        <f>2.5</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="G8" s="14" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Angle subtotal</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="16">
+        <f>SUM(E7:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
+        <f>SUM(F7:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="15" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>M.S Flat 65X6 mm</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="11">
+        <f>2.0</f>
+        <v/>
+      </c>
+      <c r="E10" s="11">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="G10" s="12" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Flat subtotal</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="16">
+        <f>SUM(E10:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="15">
+        <f>SUM(F10:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="15" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>DP Structure Iron (1 nos on canvas)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>Lgth(m)</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>Total(m)</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Wt(kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Cradle Guard (CG) Bracket on Pole</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Add: Wastage + Sag @ 3%</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
-      <c r="E10" s="11" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Total (incl. 3% wastage &amp; sag)</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="13" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>3.19</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>G.I. Wire 5 MM (6 SWG)</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Wt(kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Length (m)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Total (m)</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Wt (kg)</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>CG Earthing Wire on Span (40m)</t>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>M.S Channel 75X40 mm</t>
         </is>
       </c>
       <c r="C14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="11" t="inlineStr"/>
-      <c r="E14" s="11" t="inlineStr"/>
-      <c r="F14" s="11" t="n">
-        <v>9.84</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="D14" s="11">
+        <f>2.5</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="G14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Channel subtotal</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="16">
+        <f>SUM(E14:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>SUM(F14:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="15" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Earthing on New HT Pole (1 nos)</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>M.S Flat 65X6 mm</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="11" t="inlineStr"/>
-      <c r="E15" s="11" t="inlineStr"/>
-      <c r="F15" s="11" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Add: Wastage + Sag @ 3%</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr"/>
-      <c r="D16" s="11" t="inlineStr"/>
-      <c r="E16" s="11" t="inlineStr"/>
-      <c r="F16" s="11" t="n">
-        <v>0.39</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Total (incl. 3% wastage &amp; sag)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="inlineStr"/>
-      <c r="F17" s="13" t="n">
-        <v>13.23</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>G</t>
+      <c r="D16" s="13">
+        <f>1.0</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Flat subtotal</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="16">
+        <f>SUM(E16:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>SUM(F16:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="15" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>G.I. Wire 4 MM (8 SWG)</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
+          <t>HT Pole Iron (2 nos on canvas)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr"/>
-      <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Wt(kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Length (m)</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Total (m)</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Wt (kg)</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>CG Earthing Wire on Span (40m)</t>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>HT Single Pole (Flat - 2 nos)</t>
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="11" t="inlineStr"/>
-      <c r="E20" s="11" t="inlineStr"/>
-      <c r="F20" s="11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Add: Wastage + Sag @ 3%</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr"/>
-      <c r="D21" s="11" t="inlineStr"/>
-      <c r="E21" s="11" t="inlineStr"/>
-      <c r="F21" s="11" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Total (incl. 3% wastage &amp; sag)</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="inlineStr"/>
-      <c r="F22" s="13" t="n">
-        <v>4.12</v>
+      <c r="D20" s="11">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="E20" s="11">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G20" s="12" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="17" t="n"/>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>SECTION SUMMARY</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>M.S. Channel 100x50mm</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>9.8 kg/m</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="G23" s="18" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>M.S. Channel 75x40mm</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>6.8 kg/m</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="G24" s="18" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>M.S. Angle 65x65x6mm</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>17.25</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>5.8 kg/m</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>100.05</v>
+      </c>
+      <c r="G25" s="18" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>M.S. Flat 65x6mm</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>3.1 kg/m</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="G26" s="18" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Sub-total (all iron):</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15">
+        <f>SUM(F23:F26)</f>
+        <v/>
+      </c>
+      <c r="G28" s="15" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Add: Wastage + Sag @ 3%:</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15">
+        <f>ROUND(F28*0.03, 2)</f>
+        <v/>
+      </c>
+      <c r="G29" s="15" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="20" t="n"/>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL:</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
+      <c r="F30" s="20">
+        <f>F28+F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="20">
+        <f>CONCATENATE("=  ", FIXED(F30/1000, 4), " MT")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated base year esc bug
</commit_message>
<xml_diff>
--- a/ERP_Estimate.xlsx
+++ b/ERP_Estimate.xlsx
@@ -17,12 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0000  &quot;MT&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.000 &quot;MT&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,6 +80,12 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -217,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -248,28 +253,35 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -637,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -654,7 +666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Subject:   |  Type: NSC  |  Date: 19-05-2026</t>
+          <t>Subject:   |  Type: NSC  |  Date: 20-05-2026</t>
         </is>
       </c>
     </row>
@@ -720,11 +732,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>P C C POLE:8 Mtrs.Long</t>
+          <t>PCC POLE: 8M LONG</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -732,7 +744,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>5363.44</v>
+        <v>5293.69</v>
       </c>
       <c r="G6" s="4">
         <f>ROUND(D6*F6, 2)</f>
@@ -750,11 +762,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>G.I. Earth Spike 1833X20MM</t>
+          <t>G I EARTH SPIKE 1853X20MM</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -762,7 +774,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>367.98</v>
+        <v>465.88</v>
       </c>
       <c r="G7" s="4">
         <f>ROUND(D7*F7, 2)</f>
@@ -780,11 +792,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>G.I. Wire 5 MM (6 SWG)</t>
+          <t>G.I. WIRE 5 MM</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.006</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -792,7 +804,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>136865.98</v>
+        <v>80107.31</v>
       </c>
       <c r="G8" s="4">
         <f>ROUND(D8*F8, 2)</f>
@@ -810,7 +822,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>G.I. Stay Set LT (1680X16MM) WRKG LD-5100KG</t>
+          <t>GI STAY SET LT(1680X16MM)WRKG LD-5100KG</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -822,7 +834,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>462.17</v>
+        <v>580.51</v>
       </c>
       <c r="G9" s="4">
         <f>ROUND(D9*F9, 2)</f>
@@ -840,7 +852,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>G.I. Stay Wire 7/2.5MM (12 SWG)</t>
+          <t>G.I. STAY WIRE 7/ 2.5MM (12 SWG)</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
@@ -852,7 +864,7 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>145404.64</v>
+        <v>86748.14</v>
       </c>
       <c r="G10" s="4">
         <f>ROUND(D10*F10, 2)</f>
@@ -870,7 +882,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Porcelain Guy Insulator LT</t>
+          <t>PORCELAIN GUY INSULATOR LT</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -882,7 +894,7 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>18.37</v>
+        <v>17.64</v>
       </c>
       <c r="G11" s="4">
         <f>ROUND(D11*F11, 2)</f>
@@ -900,11 +912,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LT Distribution Box 3Ph with Steel Strap &amp; Buckle ABC</t>
+          <t>LTDISTBOX 3PH CON.WH ST.STRAP&amp;BUCKLE-ABC</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -912,7 +924,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1632.58</v>
+        <v>1499.51</v>
       </c>
       <c r="G12" s="4">
         <f>ROUND(D12*F12, 2)</f>
@@ -930,11 +942,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>IPC for ABC to ABC TEE Joint</t>
+          <t>INSULATION-PIERCING CONNECTOR -ABC TO ABC TEE JOINT</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -942,7 +954,7 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>149.17</v>
+        <v>114.95</v>
       </c>
       <c r="G13" s="4">
         <f>ROUND(D13*F13, 2)</f>
@@ -960,7 +972,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dead End Clamp LT ABC (3X70+1X16+1X50SQMM)</t>
+          <t>DEAD END CLAMP-LT ABC(3X70+1X16+1X50SMM)</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -972,7 +984,7 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>307.84</v>
+        <v>340.09</v>
       </c>
       <c r="G14" s="4">
         <f>ROUND(D14*F14, 2)</f>
@@ -990,11 +1002,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eye Hook for Anchor/Suspension Clamp</t>
+          <t>EYE HOOK FOR ANCHOR &amp; SUSPN. CLAMP</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1002,7 +1014,7 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>100.67</v>
+        <v>92.38</v>
       </c>
       <c r="G15" s="4">
         <f>ROUND(D15*F15, 2)</f>
@@ -1015,24 +1027,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0505030641</t>
+          <t>0102010611</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Suspension Clamp with Bracket 35SQMM Messenger</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>1</v>
+          <t>M.S CHANNEL 75X40 MM</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.024</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>352.89</v>
+        <v>87847.78</v>
       </c>
       <c r="G16" s="4">
         <f>ROUND(D16*F16, 2)</f>
@@ -1045,24 +1057,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0501030421</t>
+          <t>0103011511</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LT AB CABLE 1.1KV 3CX50+1CX16+1CX35SQMM</t>
+          <t>M.S FLAT 65X6 MM</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.08</v>
+        <v>0.008</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KM</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>237394.49</v>
+        <v>105704.06</v>
       </c>
       <c r="G17" s="4">
         <f>ROUND(D17*F17, 2)</f>
@@ -1075,24 +1087,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0103011511</t>
+          <t>0501030421</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>M.S Flat 65X6 mm</t>
+          <t>LT AB CABLE 1.1KV 3CX50+1CX16+1CX35SQMM</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.04</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>117493.74</v>
+        <v>237394.49</v>
       </c>
       <c r="G18" s="4">
         <f>ROUND(D18*F18, 2)</f>
@@ -1120,7 +1132,7 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Add: Escalation @ 5% for FY 24-25</t>
+          <t>Add: Sundries @ 5%</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1134,94 +1146,124 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Add: Escalation @ 5% for FY 25-26</t>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL MATERIAL COST (A)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" s="4">
-        <f>ROUND((G19+G20)*0.05, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Add: Escalation @ 5% for FY 26-27</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" s="4">
-        <f>ROUND((G19+G20+G21)*0.05, 2)</f>
+      <c r="G21" s="6">
+        <f>ROUND(G19+G20, 2)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Add: Sundries @ 5%</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" s="4">
-        <f>ROUND((G19+G20+G21+G22)*0.05, 2)</f>
-        <v/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>B. ERECTION / LABOR</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" t="n">
+        <v>1</v>
+      </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL MATERIAL COST (A)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" s="6">
-        <f>ROUND(G19+G20+G21+G22+G23, 2)</f>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Erection of 8MTR PCC Pole (LT) Without Painted</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1501</v>
+      </c>
+      <c r="G24" s="4">
+        <f>ROUND(D24*F24, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pole GIS Survey</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="G25" s="4">
+        <f>ROUND(D25*F25, 2)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>B. ERECTION / LABOR</t>
-        </is>
+      <c r="A26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Earthing Complete</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>313</v>
+      </c>
+      <c r="G26" s="4">
+        <f>ROUND(D26*F26, 2)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Erection of 8MTR PCC Pole (LT) Without Painted</t>
+          <t>LT Stay Set Complete Labour</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>SET</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>1501</v>
+        <v>555</v>
       </c>
       <c r="G27" s="4">
         <f>ROUND(D27*F27, 2)</f>
@@ -1230,16 +1272,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pole GIS Survey</t>
+          <t>Erection of Distribution Box LT ABC</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1247,7 +1289,7 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>31</v>
+        <v>507</v>
       </c>
       <c r="G28" s="4">
         <f>ROUND(D28*F28, 2)</f>
@@ -1256,16 +1298,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Earthing Complete</t>
+          <t>Fixing of IPC Connector LT ABC</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1273,7 +1315,7 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>313</v>
+        <v>75</v>
       </c>
       <c r="G29" s="4">
         <f>ROUND(D29*F29, 2)</f>
@@ -1282,12 +1324,12 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LT Stay Set Complete Labour</t>
+          <t>Erection of Anchor/Dead End Clamp LT ABC</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1295,11 +1337,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>555</v>
+        <v>154</v>
       </c>
       <c r="G30" s="4">
         <f>ROUND(D30*F30, 2)</f>
@@ -1308,24 +1350,24 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Erection of Distribution Box LT ABC</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>3</v>
+          <t>Stringing &amp; Sagging LT AB Cable 3CX50+1CX16+1CX35</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0.04</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>507</v>
+        <v>46000</v>
       </c>
       <c r="G31" s="4">
         <f>ROUND(D31*F31, 2)</f>
@@ -1334,24 +1376,24 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fixing of IPC Connector LT ABC</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>12</v>
+          <t>Survey for L.T.O.H Line</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>0.04</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>75</v>
+        <v>1714</v>
       </c>
       <c r="G32" s="4">
         <f>ROUND(D32*F32, 2)</f>
@@ -1359,209 +1401,105 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
-        <v>7</v>
-      </c>
+      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Erection of Anchor/Dead End Clamp LT ABC</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>154</v>
-      </c>
-      <c r="G33" s="4">
-        <f>ROUND(D33*F33, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>8</v>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Erection of Suspension Clamp LT ABC</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>154</v>
-      </c>
-      <c r="G34" s="4">
-        <f>ROUND(D34*F34, 2)</f>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL LABOR COST (B)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" s="6">
+        <f>ROUND(SUM(G24:G32), 2)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>9</v>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Stringing &amp; Sagging LT AB Cable 3CX50+1CX16+1CX35</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>KM</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>46000</v>
-      </c>
-      <c r="G35" s="4">
-        <f>ROUND(D35*F35, 2)</f>
-        <v/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>C. OVERHEADS &amp; TAXES</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>10</v>
-      </c>
+      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Survey for L.T.O.H Line</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>KM</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>1714</v>
-      </c>
+          <t>Supervision @ 10% on (A+B)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" s="4">
-        <f>ROUND(D36*F36, 2)</f>
+        <f>ROUND((G21+G33)*0.1, 2)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL LABOR COST (B)</t>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GST @ 18% on Labour only</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" s="6">
-        <f>ROUND(SUM(G27:G36), 2)</f>
+      <c r="G37" s="4">
+        <f>ROUND(G33*0.18, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sub-Total</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" s="4">
+        <f>ROUND(G21+G33+G36+G37, 2)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>C. OVERHEADS &amp; TAXES</t>
-        </is>
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Add: Cess @ 1% on (Mat+Lab+Sup)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" s="4">
+        <f>ROUND((G21+G33+G36)*0.01, 2)</f>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Supervision @ 10% on (A+B)</t>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" s="4">
-        <f>ROUND((G24+G37)*0.1, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>GST @ 18% on Labour only</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" s="4">
-        <f>ROUND(G37*0.18, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Sub-Total</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" s="4">
-        <f>ROUND(G24+G37+G40+G41, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Add: Cess @ 1% on (Mat+Lab+Sup)</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" s="4">
-        <f>ROUND((G24+G37+G40)*0.01, 2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" s="8">
-        <f>ROUND(G42+G43, 2)</f>
+      <c r="G40" s="8">
+        <f>ROUND(G38+G39, 2)</f>
         <v/>
       </c>
     </row>
@@ -1581,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1655,7 +1593,7 @@
       <c r="A4" s="16" t="n"/>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳  LT Pole Iron — LT Pole Iron Recipe  (3 nos on canvas)</t>
+          <t xml:space="preserve">  ↳  LT Pole Iron — LT Pole Iron Recipe  (2 nos on canvas)</t>
         </is>
       </c>
       <c r="C4" s="14" t="n"/>
@@ -1673,7 +1611,7 @@
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="18">
         <f>1.5+0.3</f>
@@ -1717,7 +1655,7 @@
       <c r="D7" s="24" t="n"/>
       <c r="E7" s="24" t="n"/>
       <c r="F7" s="25">
-        <f>ROUND(F6,4)</f>
+        <f>ROUND(F6,3)</f>
         <v/>
       </c>
     </row>
@@ -1745,7 +1683,7 @@
       <c r="A10" s="16" t="n"/>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳  LT Pole Iron — LT Pole Iron Recipe  (3 nos on canvas)</t>
+          <t xml:space="preserve">  ↳  LT Pole Iron — LT Pole Iron Recipe  (2 nos on canvas)</t>
         </is>
       </c>
       <c r="C10" s="14" t="n"/>
@@ -1763,7 +1701,7 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="18">
         <f>1</f>
@@ -1800,7 +1738,7 @@
       <c r="A13" s="16" t="n"/>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳  AB Cable Clamp (2 spans)  (2 nos on canvas)</t>
+          <t xml:space="preserve">  ↳  AB Cable Clamp (1 spans)  (1 nos on canvas)</t>
         </is>
       </c>
       <c r="C13" s="14" t="n"/>
@@ -1818,7 +1756,7 @@
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="18">
         <f>0.5</f>
@@ -1837,7 +1775,7 @@
       <c r="A15" s="21" t="n"/>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Iron Total — AB Cable Clamp (2 spans)</t>
+          <t xml:space="preserve">  Iron Total — AB Cable Clamp (1 spans)</t>
         </is>
       </c>
       <c r="C15" s="21" t="n"/>
@@ -1862,59 +1800,95 @@
       <c r="D16" s="24" t="n"/>
       <c r="E16" s="24" t="n"/>
       <c r="F16" s="25">
-        <f>ROUND(F12+F15,4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="26" t="n"/>
-      <c r="B19" s="26" t="inlineStr">
+        <f>ROUND(F12+F15,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>IRON SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>M.S. Channel (75X40mm)</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="28" t="n">
+        <v>0.024</v>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="27" t="n"/>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>M.S. Flat (65X6mm)</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="28" t="n">
+        <v>0.008</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="29" t="n"/>
+      <c r="B23" s="29" t="inlineStr">
         <is>
           <t>TOTAL IRON (as per Estimate):</t>
         </is>
       </c>
-      <c r="C19" s="26" t="n"/>
-      <c r="D19" s="26" t="n"/>
-      <c r="E19" s="26" t="n"/>
-      <c r="F19" s="27">
-        <f>ROUND(F7+F16,4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="28" t="n"/>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="29" t="n"/>
+      <c r="F23" s="30">
+        <f>ROUND(F20+F21,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="31" t="n"/>
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Add: Fabrication Wastage @ 3%:</t>
         </is>
       </c>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="29">
-        <f>ROUND(F19*0.03,4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="30" t="n"/>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>TOTAL FOR PROCUREMENT (incl. 3% wastage):</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="n"/>
-      <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
-      <c r="F21" s="31">
-        <f>ROUND(F19+F20,4)</f>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="31" t="n"/>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="32">
+        <f>ROUND(F23*0.03,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="33" t="n"/>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL IRON (incl. wastage):</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="33" t="n"/>
+      <c r="E25" s="33" t="n"/>
+      <c r="F25" s="34">
+        <f>ROUND(F23+F24,3)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B3:E3"/>

</xml_diff>